<commit_message>
update databasing for archive
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level0_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level0_nirda.xlsx
@@ -1572,12 +1572,12 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>JSgZKRZWJRfWJRZW</t>
+          <t>LUeYORbXLRbXLRbX</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-01-08T14:08:01</t>
+          <t>HDU checksum updated 2026-01-16T10:20:00</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-01-08T14:08:01</t>
+          <t>data unit checksum updated 2026-01-16T10:20:00</t>
         </is>
       </c>
     </row>
@@ -1846,12 +1846,12 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>eEZ6gCX6eCX6eCX6</t>
+          <t>hDa8hDU6hDa6hDU6</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-01-08T14:08:02</t>
+          <t>HDU checksum updated 2026-01-16T10:20:01</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-01-08T14:08:02</t>
+          <t>data unit checksum updated 2026-01-16T10:20:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update hacks for rae
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level0_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level0_nirda.xlsx
@@ -766,7 +766,7 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>v2.08</t>
+          <t>v3.03</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -802,7 +802,7 @@
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -818,7 +818,11 @@
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>HAT-P-26b</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Target ID/keyword</t>
@@ -834,7 +838,7 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>/sssp/data/2025/04/05/2025-04-05__13-15-18_InfImg_d2048x2048x0050_b1_e01_i01_g01_d00_r50.sp</t>
+          <t>/sssp/data/2026/04/01/2026-04-01__00-03-18_InfImg_HAT-P-26b_d0200x0600x0472_b1_e01_i59_g02_d16_r04.sp</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -906,7 +910,7 @@
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1610</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -924,7 +928,7 @@
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>750</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -960,7 +964,7 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -978,7 +982,7 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>600</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -996,7 +1000,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>118</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1032,7 +1036,7 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>28</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1050,7 +1054,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>797174156</t>
+          <t>828317035</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1068,7 +1072,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>738000000</t>
+          <t>818000000</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1230,7 +1234,7 @@
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1266,7 +1270,7 @@
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1284,7 +1288,7 @@
       <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1302,7 +1306,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>59</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1392,7 +1396,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>1475</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1410,7 +1414,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>472</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1428,7 +1432,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>472</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1446,7 +1450,7 @@
       <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1464,7 +1468,7 @@
       <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>5.65685</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1482,7 +1486,7 @@
       <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10736</t>
+          <t>1276</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1500,7 +1504,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>999.0</t>
+          <t>-2.6456665992736816</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1518,7 +1522,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>297.6682434082031</t>
+          <t>264.48187255859375</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1536,7 +1540,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>78.88285064697266</t>
+          <t>138.0994873046875</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1554,7 +1558,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>68.87708282470703</t>
+          <t>127.01375579833984</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1572,12 +1576,12 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LQdXNPbULPbULPbU</t>
+          <t>GY7FIW79GW7CGW79</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-01-16T15:40:13</t>
+          <t>HDU checksum updated 2026-04-08T14:21:24</t>
         </is>
       </c>
     </row>
@@ -1595,7 +1599,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-01-16T15:40:13</t>
+          <t>data unit checksum updated 2026-04-08T14:21:24</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1714,7 @@
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>200</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
@@ -1724,7 +1728,7 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2048</t>
+          <t>600</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -1738,7 +1742,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>118</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -1846,12 +1850,12 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>gBa6jAV3gAZ3gAZ3</t>
+          <t>WEfAa9d3YCdAa9d3</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-01-16T15:40:15</t>
+          <t>HDU checksum updated 2026-04-08T14:21:24</t>
         </is>
       </c>
     </row>
@@ -1864,12 +1868,12 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1494830781</t>
+          <t>2131261651</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-01-16T15:40:15</t>
+          <t>data unit checksum updated 2026-04-08T14:21:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update for soc report
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level0_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level0_nirda.xlsx
@@ -1576,12 +1576,12 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>oi2Uqg1Sog1Sog1S</t>
+          <t>0h2U1f2R0f2R0f2R</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-08-25T21:26:25</t>
+          <t>HDU checksum updated 2026-09-08T14:41:25</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-08-25T21:26:25</t>
+          <t>data unit checksum updated 2026-09-08T14:41:25</t>
         </is>
       </c>
     </row>
@@ -1850,12 +1850,12 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LZYaOYWULYWaLYWU</t>
+          <t>MYYZOXXZMXXZMXXZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-08-25T21:26:25</t>
+          <t>HDU checksum updated 2026-09-08T14:41:25</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-08-25T21:26:25</t>
+          <t>data unit checksum updated 2026-09-08T14:41:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated inspector for easier dev
</commit_message>
<xml_diff>
--- a/src/pandorafits/formats/nirda/level0_nirda.xlsx
+++ b/src/pandorafits/formats/nirda/level0_nirda.xlsx
@@ -820,7 +820,7 @@
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HD_200654</t>
+          <t>KELT-9b</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -838,7 +838,7 @@
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
-          <t>/sssp/data/2026/08/15/2026-08-15__03-03-20_InfImg_HD_200654_d0080x0250x1583_b1_e01_i427_g02_d16_r04.sp</t>
+          <t>/sssp/data/2026/08/15/2026-08-15__06-44-18_InfImg_KELT-9b_d0080x0250x3096_b1_e01_i387_g02_d16_r04.sp</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1000,7 +1000,7 @@
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>394</t>
+          <t>774</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1054,7 +1054,7 @@
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
-          <t>840078241</t>
+          <t>840091495</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1072,7 +1072,7 @@
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
-          <t>877000000</t>
+          <t>832000000</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1306,7 +1306,7 @@
       <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>387</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1396,7 +1396,7 @@
       <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
-          <t>11360</t>
+          <t>10320</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1414,7 +1414,7 @@
       <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3416</t>
+          <t>3096</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1432,7 +1432,7 @@
       <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
-          <t>1583</t>
+          <t>3096</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1504,7 +1504,7 @@
       <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
-          <t>0.5968567132949829</t>
+          <t>3.3816466331481934</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1522,7 +1522,7 @@
       <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
-          <t>276.0766906738281</t>
+          <t>278.990966796875</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -1540,7 +1540,7 @@
       <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
-          <t>131.3281707763672</t>
+          <t>131.50372314453125</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -1558,7 +1558,7 @@
       <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
-          <t>120.02909851074219</t>
+          <t>120.03438568115234</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -1576,12 +1576,12 @@
       <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0h2U1f2R0f2R0f2R</t>
+          <t>08m736k506k506k5</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-09-08T14:41:25</t>
+          <t>HDU checksum updated 2026-09-09T15:45:53</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-09-08T14:41:25</t>
+          <t>data unit checksum updated 2026-09-09T15:45:53</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>394</t>
+          <t>774</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -1850,12 +1850,12 @@
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MYYZOXXZMXXZMXXZ</t>
+          <t>oDGar9FVoCFZo9FZ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>HDU checksum updated 2026-09-08T14:41:25</t>
+          <t>HDU checksum updated 2026-09-09T15:45:53</t>
         </is>
       </c>
     </row>
@@ -1868,12 +1868,12 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>4231325753</t>
+          <t>1450830242</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>data unit checksum updated 2026-09-08T14:41:25</t>
+          <t>data unit checksum updated 2026-09-09T15:45:53</t>
         </is>
       </c>
     </row>

</xml_diff>